<commit_message>
Complete HW2 model anatomy assignment
</commit_message>
<xml_diff>
--- a/hw2/docs/anatomy-worksheet.xlsx
+++ b/hw2/docs/anatomy-worksheet.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как пользоваться" sheetId="1" r:id="R6caaf5ed43324654"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Параметры" sheetId="2" r:id="Rd22b19b3ee0b4320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoRA" sheetId="3" r:id="R1e52045654474dca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Память" sheetId="4" r:id="R158d9e8e813d464f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ответы" sheetId="5" r:id="R4597aa232bf8409a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как пользоваться" sheetId="1" r:id="R80babf8d301a471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Параметры" sheetId="2" r:id="R8bf3d1bcbda64444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoRA" sheetId="3" r:id="R5ff819aeb3dd4b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Память" sheetId="4" r:id="R31c21a691cf546ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ответы" sheetId="5" r:id="R265a22ac0ace404a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,16 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="7">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="164" formatCode="0.000%"/>
     <x:numFmt numFmtId="165" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="166" formatCode="0.0"/>
-    <x:numFmt numFmtId="200" formatCode="#,##0"/>
-    <x:numFmt numFmtId="201" formatCode="General"/>
-    <x:numFmt numFmtId="202" formatCode="0.00%"/>
-    <x:numFmt numFmtId="203" formatCode="0.000"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -60,51 +56,13 @@
       <x:color rgb="FF1A1A2E"/>
       <x:name val="Consolas"/>
     </x:font>
-    <x:font>
-      <x:i/>
-      <x:sz val="10"/>
-      <x:color rgb="FF8888AA"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color theme="1"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="14"/>
-      <x:color rgb="FF7E22CE"/>
-      <x:name val="Calibri"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE9D5FF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF9E6"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF5F0FF"/>
-      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -166,7 +124,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="89">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -200,161 +158,11 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="3" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="10" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="202" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="202" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="202" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="202" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="166" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="166" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="203" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="2">
     <x:dxf>
       <x:fill>
         <x:patternFill>
@@ -366,20 +174,6 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="00DCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDCFCE7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -818,7 +612,7 @@
     <x:col min="6" max="6" width="18" customWidth="1"/>
     <x:col min="7" max="7" width="14" customWidth="1"/>
     <x:col min="8" max="8" width="12" customWidth="1"/>
-    <x:col min="9" max="9" width="47" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -835,7 +629,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="4" ht="52" customHeight="1">
+    <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">модуль</x:t>
@@ -898,22 +692,22 @@
       <x:c r="D5" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E5" s="35" t="n">
+      <x:c r="E5" s="9" t="n">
         <x:f>IF(COUNT(B5:D5)=3,B5*C5*D5,"")</x:f>
         <x:v>155582464</x:v>
       </x:c>
-      <x:c r="F5" s="36" t="n">
+      <x:c r="F5" s="10" t="n">
         <x:v>155582464</x:v>
       </x:c>
       <x:c r="G5" s="11" t="str">
         <x:f>IF(E5="","—",IF(E5=F5,"сходится","РАСХОЖДЕНИЕ"))</x:f>
         <x:v>сходится</x:v>
       </x:c>
-      <x:c r="H5" s="42" t="n">
+      <x:c r="H5" s="12" t="n">
         <x:f>IF($F$15=0,"",F5/$F$15)</x:f>
         <x:v>0.2610225398570643</x:v>
       </x:c>
-      <x:c r="I5" s="25" t="inlineStr">
+      <x:c r="I5" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -934,22 +728,22 @@
       <x:c r="D6" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E6" s="35" t="n">
+      <x:c r="E6" s="9" t="n">
         <x:f>IF(COUNT(B6:D6)=3,B6*C6*D6,"")</x:f>
         <x:v>58720256</x:v>
       </x:c>
-      <x:c r="F6" s="36" t="n">
+      <x:c r="F6" s="10" t="n">
         <x:v>58720256</x:v>
       </x:c>
       <x:c r="G6" s="11" t="str">
         <x:f>IF(E6="","—",IF(E6=F6,"сходится","РАСХОЖДЕНИЕ"))</x:f>
         <x:v>сходится</x:v>
       </x:c>
-      <x:c r="H6" s="42" t="n">
+      <x:c r="H6" s="12" t="n">
         <x:f>IF($F$15=0,"",F6/$F$15)</x:f>
         <x:v>0.09851566794942276</x:v>
       </x:c>
-      <x:c r="I6" s="25" t="inlineStr">
+      <x:c r="I6" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -970,22 +764,22 @@
       <x:c r="D7" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E7" s="35" t="n">
+      <x:c r="E7" s="9" t="n">
         <x:f>IF(COUNT(B7:D7)=3,B7*C7*D7,"")</x:f>
         <x:v>29360128</x:v>
       </x:c>
-      <x:c r="F7" s="36" t="n">
+      <x:c r="F7" s="10" t="n">
         <x:v>29360128</x:v>
       </x:c>
       <x:c r="G7" s="11" t="str">
         <x:f>IF(E7="","—",IF(E7=F7,"сходится","РАСХОЖДЕНИЕ"))</x:f>
         <x:v>сходится</x:v>
       </x:c>
-      <x:c r="H7" s="42" t="n">
+      <x:c r="H7" s="12" t="n">
         <x:f>IF($F$15=0,"",F7/$F$15)</x:f>
         <x:v>0.04925783397471138</x:v>
       </x:c>
-      <x:c r="I7" s="25" t="inlineStr">
+      <x:c r="I7" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -1006,22 +800,22 @@
       <x:c r="D8" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E8" s="35" t="n">
+      <x:c r="E8" s="9" t="n">
         <x:f>IF(COUNT(B8:D8)=3,B8*C8*D8,"")</x:f>
         <x:v>29360128</x:v>
       </x:c>
-      <x:c r="F8" s="36" t="n">
+      <x:c r="F8" s="10" t="n">
         <x:v>29360128</x:v>
       </x:c>
       <x:c r="G8" s="11" t="str">
         <x:f>IF(E8="","—",IF(E8=F8,"сходится","РАСХОЖДЕНИЕ"))</x:f>
         <x:v>сходится</x:v>
       </x:c>
-      <x:c r="H8" s="42" t="n">
+      <x:c r="H8" s="12" t="n">
         <x:f>IF($F$15=0,"",F8/$F$15)</x:f>
         <x:v>0.04925783397471138</x:v>
       </x:c>
-      <x:c r="I8" s="25" t="inlineStr">
+      <x:c r="I8" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -1042,22 +836,22 @@
       <x:c r="D9" s="8" t="n">
         <x:v>2048</x:v>
       </x:c>
-      <x:c r="E9" s="35" t="n">
+      <x:c r="E9" s="9" t="n">
         <x:f>IF(COUNT(B9:D9)=3,B9*C9*D9,"")</x:f>
         <x:v>58720256</x:v>
       </x:c>
-      <x:c r="F9" s="36" t="n">
+      <x:c r="F9" s="10" t="n">
         <x:v>58720256</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
         <x:f>IF(E9="","—",IF(E9=F9,"сходится","РАСХОЖДЕНИЕ"))</x:f>
         <x:v>сходится</x:v>
       </x:c>
-      <x:c r="H9" s="42" t="n">
+      <x:c r="H9" s="12" t="n">
         <x:f>IF($F$15=0,"",F9/$F$15)</x:f>
         <x:v>0.09851566794942276</x:v>
       </x:c>
-      <x:c r="I9" s="25" t="inlineStr">
+      <x:c r="I9" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -1078,22 +872,22 @@
       <x:c r="D10" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E10" s="35" t="n">
+      <x:c r="E10" s="9" t="n">
         <x:f>IF(COUNT(B10:D10)=3,B10*C10*D10,"")</x:f>
         <x:v>88080384</x:v>
       </x:c>
-      <x:c r="F10" s="36" t="n">
+      <x:c r="F10" s="10" t="n">
         <x:v>88080384</x:v>
       </x:c>
       <x:c r="G10" s="11" t="str">
         <x:f>IF(E10="","—",IF(E10=F10,"сходится","РАСХОЖДЕНИЕ"))</x:f>
         <x:v>сходится</x:v>
       </x:c>
-      <x:c r="H10" s="42" t="n">
+      <x:c r="H10" s="12" t="n">
         <x:f>IF($F$15=0,"",F10/$F$15)</x:f>
         <x:v>0.14777350192413413</x:v>
       </x:c>
-      <x:c r="I10" s="25" t="inlineStr">
+      <x:c r="I10" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -1114,22 +908,22 @@
       <x:c r="D11" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E11" s="35" t="n">
+      <x:c r="E11" s="9" t="n">
         <x:f>IF(COUNT(B11:D11)=3,B11*C11*D11,"")</x:f>
         <x:v>88080384</x:v>
       </x:c>
-      <x:c r="F11" s="36" t="n">
+      <x:c r="F11" s="10" t="n">
         <x:v>88080384</x:v>
       </x:c>
       <x:c r="G11" s="11" t="str">
         <x:f>IF(E11="","—",IF(E11=F11,"сходится","РАСХОЖДЕНИЕ"))</x:f>
         <x:v>сходится</x:v>
       </x:c>
-      <x:c r="H11" s="42" t="n">
+      <x:c r="H11" s="12" t="n">
         <x:f>IF($F$15=0,"",F11/$F$15)</x:f>
         <x:v>0.14777350192413413</x:v>
       </x:c>
-      <x:c r="I11" s="25" t="inlineStr">
+      <x:c r="I11" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
@@ -1150,93 +944,87 @@
       <x:c r="D12" s="8" t="n">
         <x:v>3072</x:v>
       </x:c>
-      <x:c r="E12" s="35" t="n">
+      <x:c r="E12" s="9" t="n">
         <x:f>IF(COUNT(B12:D12)=3,B12*C12*D12,"")</x:f>
         <x:v>88080384</x:v>
       </x:c>
-      <x:c r="F12" s="36" t="n">
+      <x:c r="F12" s="10" t="n">
         <x:v>88080384</x:v>
       </x:c>
       <x:c r="G12" s="11" t="str">
         <x:f>IF(E12="","—",IF(E12=F12,"сходится","РАСХОЖДЕНИЕ"))</x:f>
         <x:v>сходится</x:v>
       </x:c>
-      <x:c r="H12" s="42" t="n">
+      <x:c r="H12" s="12" t="n">
         <x:f>IF($F$15=0,"",F12/$F$15)</x:f>
         <x:v>0.14777350192413413</x:v>
       </x:c>
-      <x:c r="I12" s="25" t="inlineStr">
+      <x:c r="I12" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="13" ht="32" customHeight="1">
-      <x:c r="A13" s="27" t="inlineStr">
+    <x:row r="13">
+      <x:c r="A13" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">norm</x:t>
         </x:is>
       </x:c>
-      <x:c r="B13" s="28" t="n">
+      <x:c r="B13" s="8" t="n">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="C13" s="28" t="str">
-        <x:v>128 / 1024</x:v>
-      </x:c>
-      <x:c r="D13" s="28" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E13" s="37" t="n">
-        <x:f>SUM(E22:E23)</x:f>
+      <x:c r="C13" s="8"/>
+      <x:c r="D13" s="8"/>
+      <x:c r="E13" s="9" t="str">
+        <x:f>IF(COUNT(B13:D13)=3,B13*C13*D13,"")</x:f>
+      </x:c>
+      <x:c r="F13" s="10" t="n">
         <x:v>65536</x:v>
       </x:c>
-      <x:c r="F13" s="38" t="n">
-        <x:v>65536</x:v>
-      </x:c>
-      <x:c r="G13" s="31" t="str">
+      <x:c r="G13" s="11" t="str">
         <x:f>IF(E13="","—",IF(E13=F13,"сходится","РАСХОЖДЕНИЕ"))</x:f>
-        <x:v>сходится</x:v>
-      </x:c>
-      <x:c r="H13" s="43" t="n">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H13" s="12" t="n">
         <x:f>IF($F$15=0,"",F13/$F$15)</x:f>
         <x:v>0.00010995052226498076</x:v>
       </x:c>
-      <x:c r="I13" s="34" t="str">
-        <x:v>56×128 + 57×1024; см. расчёт ниже.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="32" customHeight="1">
-      <x:c r="A14" s="27" t="inlineStr">
+      <x:c r="I13" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">вектор, а не матрица: столбцов нет</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">lm_head</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" s="28" t="n">
+      <x:c r="B14" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C14" s="28" t="n">
-        <x:v>151936</x:v>
-      </x:c>
-      <x:c r="D14" s="28" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="E14" s="37" t="n">
-        <x:f>B14*C14*D14-F5</x:f>
+      <x:c r="C14" s="8"/>
+      <x:c r="D14" s="8"/>
+      <x:c r="E14" s="9" t="str">
+        <x:f>IF(COUNT(B14:D14)=3,B14*C14*D14,"")</x:f>
+      </x:c>
+      <x:c r="F14" s="10" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F14" s="38" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G14" s="31" t="str">
-        <x:f>IF(COUNT(E14)=0,"—",IF(E14=F14,"сходится","РАСХОЖДЕНИЕ"))</x:f>
-        <x:v>сходится</x:v>
-      </x:c>
-      <x:c r="H14" s="43" t="n">
+      <x:c r="G14" s="11" t="str">
+        <x:f>IF(E14="","—",IF(E14=F14,"сходится","РАСХОЖДЕНИЕ"))</x:f>
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H14" s="12" t="n">
         <x:f>IF($F$15=0,"",F14/$F$15)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I14" s="34" t="str">
-        <x:v>Общий тензор с embed; собственных весов нет.</x:v>
+      <x:c r="I14" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">tie_word_embeddings — своих весов нет</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1245,22 +1033,14 @@
           <x:t xml:space="preserve">ИТОГО</x:t>
         </x:is>
       </x:c>
-      <x:c r="E15" s="39"/>
-      <x:c r="F15" s="40" t="n">
+      <x:c r="F15" s="15" t="n">
         <x:f>SUM(F5:F14)</x:f>
         <x:v>596049920</x:v>
       </x:c>
-      <x:c r="H15" s="42" t="n">
+      <x:c r="H15" s="12" t="n">
         <x:f>IF(F15=0,"",F15/F15)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I15" s="26"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="E16" s="39"/>
-      <x:c r="F16" s="39"/>
-      <x:c r="H16" s="44"/>
-      <x:c r="I16" s="26"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="14" t="inlineStr">
@@ -1268,12 +1048,9 @@
           <x:t xml:space="preserve">params_total из отчёта</x:t>
         </x:is>
       </x:c>
-      <x:c r="E17" s="39"/>
-      <x:c r="F17" s="36" t="n">
+      <x:c r="F17" s="10" t="n">
         <x:v>596049920</x:v>
       </x:c>
-      <x:c r="H17" s="44"/>
-      <x:c r="I17" s="26"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="14" t="inlineStr">
@@ -1281,139 +1058,9 @@
           <x:t xml:space="preserve">сумма сошлась?</x:t>
         </x:is>
       </x:c>
-      <x:c r="E18" s="39"/>
-      <x:c r="F18" s="41" t="str">
+      <x:c r="F18" s="11" t="str">
         <x:f>IF(F17="","заполните",IF(F15=F17,"да, сходится","НЕ СХОДИТСЯ"))</x:f>
         <x:v>да, сходится</x:v>
-      </x:c>
-      <x:c r="H18" s="44"/>
-      <x:c r="I18" s="26"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="H19" s="44"/>
-      <x:c r="I19" s="26"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>Расшифровка norm: уже учтена в строке 13</x:v>
-      </x:c>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="H20" s="44"/>
-      <x:c r="I20" s="26"/>
-    </x:row>
-    <x:row r="21" ht="52" customHeight="1">
-      <x:c r="A21" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">модуль</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B21" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">штук</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C21" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">строк</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D21" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">столбцов</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E21" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">по формуле
-штук × строк × столбцов</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F21" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">по sum(p.numel())</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G21" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">сходится?</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H21" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">доля модели</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I21" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">примечание</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="59" t="str">
-        <x:v>norm 128</x:v>
-      </x:c>
-      <x:c r="B22" s="63" t="n">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="C22" s="63" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="D22" s="63" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E22" s="65" t="n">
-        <x:f>B22*C22*D22</x:f>
-        <x:v>7168</x:v>
-      </x:c>
-      <x:c r="F22" s="64" t="n">
-        <x:v>7168</x:v>
-      </x:c>
-      <x:c r="G22" s="66" t="str">
-        <x:f>IF(E22=F22,"сходится","РАСХОЖДЕНИЕ")</x:f>
-        <x:v>сходится</x:v>
-      </x:c>
-      <x:c r="H22" s="67" t="n">
-        <x:f>F22/$F$15</x:f>
-        <x:v>0.000012025838372732271</x:v>
-      </x:c>
-      <x:c r="I22" s="62" t="str">
-        <x:v>Вектор; учтён в общей строке norm</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="59" t="str">
-        <x:v>norm 1024</x:v>
-      </x:c>
-      <x:c r="B23" s="63" t="n">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="C23" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="D23" s="63" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E23" s="65" t="n">
-        <x:f>B23*C23*D23</x:f>
-        <x:v>58368</x:v>
-      </x:c>
-      <x:c r="F23" s="64" t="n">
-        <x:v>58368</x:v>
-      </x:c>
-      <x:c r="G23" s="66" t="str">
-        <x:f>IF(E23=F23,"сходится","РАСХОЖДЕНИЕ")</x:f>
-        <x:v>сходится</x:v>
-      </x:c>
-      <x:c r="H23" s="67" t="n">
-        <x:f>F23/$F$15</x:f>
-        <x:v>0.00009792468389224849</x:v>
-      </x:c>
-      <x:c r="I23" s="62" t="str">
-        <x:v>Вектор; учтён в общей строке norm</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1441,7 +1088,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" customWidth="1"/>
     <x:col min="2" max="2" width="10" customWidth="1"/>
     <x:col min="3" max="3" width="10" customWidth="1"/>
     <x:col min="4" max="4" width="10" customWidth="1"/>
@@ -1450,21 +1097,18 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>LoRA: r=8, q_proj+v_proj</x:v>
+      <x:c r="A1" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Параметры LoRA: своя формула против peft</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="70" t="inlineStr">
+      <x:c r="A2" s="5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">На каждый целевой модуль адаптер добавляет r × (вход + выход) чисел. Умножаем на число слоёв.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="71"/>
-      <x:c r="C2" s="71"/>
-      <x:c r="D2" s="71"/>
-      <x:c r="E2" s="71"/>
-      <x:c r="F2" s="71"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="14" t="inlineStr">
@@ -1486,7 +1130,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="45" customHeight="1">
+    <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">целевой модуль</x:t>
@@ -1520,8 +1164,10 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="7" t="str">
-        <x:v>q_proj</x:v>
+      <x:c r="A8" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">q_proj</x:t>
+        </x:is>
       </x:c>
       <x:c r="B8" s="8" t="n">
         <x:v>28</x:v>
@@ -1532,7 +1178,7 @@
       <x:c r="D8" s="8" t="n">
         <x:v>2048</x:v>
       </x:c>
-      <x:c r="E8" s="35" t="n">
+      <x:c r="E8" s="9" t="n">
         <x:f>IF(OR(F8&lt;&gt;"да",COUNT(B8:D8)&lt;3),0,$B$4*(C8+D8)*B8)</x:f>
         <x:v>688128</x:v>
       </x:c>
@@ -1541,8 +1187,10 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="7" t="str">
-        <x:v>k_proj</x:v>
+      <x:c r="A9" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">k_proj</x:t>
+        </x:is>
       </x:c>
       <x:c r="B9" s="8" t="n">
         <x:v>28</x:v>
@@ -1553,7 +1201,7 @@
       <x:c r="D9" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E9" s="35" t="n">
+      <x:c r="E9" s="9" t="n">
         <x:f>IF(OR(F9&lt;&gt;"да",COUNT(B9:D9)&lt;3),0,$B$4*(C9+D9)*B9)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1562,8 +1210,10 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="7" t="str">
-        <x:v>v_proj</x:v>
+      <x:c r="A10" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v_proj</x:t>
+        </x:is>
       </x:c>
       <x:c r="B10" s="8" t="n">
         <x:v>28</x:v>
@@ -1574,7 +1224,7 @@
       <x:c r="D10" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E10" s="35" t="n">
+      <x:c r="E10" s="9" t="n">
         <x:f>IF(OR(F10&lt;&gt;"да",COUNT(B10:D10)&lt;3),0,$B$4*(C10+D10)*B10)</x:f>
         <x:v>458752</x:v>
       </x:c>
@@ -1583,8 +1233,10 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="7" t="str">
-        <x:v>o_proj</x:v>
+      <x:c r="A11" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">o_proj</x:t>
+        </x:is>
       </x:c>
       <x:c r="B11" s="8" t="n">
         <x:v>28</x:v>
@@ -1595,7 +1247,7 @@
       <x:c r="D11" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E11" s="35" t="n">
+      <x:c r="E11" s="9" t="n">
         <x:f>IF(OR(F11&lt;&gt;"да",COUNT(B11:D11)&lt;3),0,$B$4*(C11+D11)*B11)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1604,8 +1256,10 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="7" t="str">
-        <x:v>gate_proj</x:v>
+      <x:c r="A12" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">gate_proj</x:t>
+        </x:is>
       </x:c>
       <x:c r="B12" s="8" t="n">
         <x:v>28</x:v>
@@ -1616,7 +1270,7 @@
       <x:c r="D12" s="8" t="n">
         <x:v>3072</x:v>
       </x:c>
-      <x:c r="E12" s="35" t="n">
+      <x:c r="E12" s="9" t="n">
         <x:f>IF(OR(F12&lt;&gt;"да",COUNT(B12:D12)&lt;3),0,$B$4*(C12+D12)*B12)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1625,8 +1279,10 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="7" t="str">
-        <x:v>up_proj</x:v>
+      <x:c r="A13" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">up_proj</x:t>
+        </x:is>
       </x:c>
       <x:c r="B13" s="8" t="n">
         <x:v>28</x:v>
@@ -1637,7 +1293,7 @@
       <x:c r="D13" s="8" t="n">
         <x:v>3072</x:v>
       </x:c>
-      <x:c r="E13" s="35" t="n">
+      <x:c r="E13" s="9" t="n">
         <x:f>IF(OR(F13&lt;&gt;"да",COUNT(B13:D13)&lt;3),0,$B$4*(C13+D13)*B13)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1646,8 +1302,10 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="7" t="str">
-        <x:v>down_proj</x:v>
+      <x:c r="A14" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">down_proj</x:t>
+        </x:is>
       </x:c>
       <x:c r="B14" s="8" t="n">
         <x:v>28</x:v>
@@ -1658,7 +1316,7 @@
       <x:c r="D14" s="8" t="n">
         <x:v>1024</x:v>
       </x:c>
-      <x:c r="E14" s="35" t="n">
+      <x:c r="E14" s="9" t="n">
         <x:f>IF(OR(F14&lt;&gt;"да",COUNT(B14:D14)&lt;3),0,$B$4*(C14+D14)*B14)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1672,7 +1330,7 @@
           <x:t xml:space="preserve">по вашей формуле</x:t>
         </x:is>
       </x:c>
-      <x:c r="E15" s="40" t="n">
+      <x:c r="E15" s="15" t="n">
         <x:f>SUM(E8:E14)</x:f>
         <x:v>1146880</x:v>
       </x:c>
@@ -1683,7 +1341,7 @@
           <x:t xml:space="preserve">что показал peft</x:t>
         </x:is>
       </x:c>
-      <x:c r="E16" s="36" t="n">
+      <x:c r="E16" s="10" t="n">
         <x:v>1146880</x:v>
       </x:c>
     </x:row>
@@ -1714,337 +1372,10 @@
           <x:t xml:space="preserve">доля обучаемых</x:t>
         </x:is>
       </x:c>
-      <x:c r="E20" s="68" t="n">
+      <x:c r="E20" s="16" t="n">
         <x:f>IF(E19="","",E15/E19)</x:f>
         <x:v>0.0019241341396371632</x:v>
       </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="73" t="str">
-        <x:v>LoRA: r=16, все линейные</x:v>
-      </x:c>
-      <x:c r="B25" s="59"/>
-      <x:c r="C25" s="59"/>
-      <x:c r="D25" s="59"/>
-      <x:c r="E25" s="59"/>
-      <x:c r="F25" s="59"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">На каждый целевой модуль адаптер добавляет r × (вход + выход) чисел. Умножаем на число слоёв.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B26" s="59"/>
-      <x:c r="C26" s="59"/>
-      <x:c r="D26" s="59"/>
-      <x:c r="E26" s="59"/>
-      <x:c r="F26" s="59"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="59"/>
-      <x:c r="B27" s="59"/>
-      <x:c r="C27" s="59"/>
-      <x:c r="D27" s="59"/>
-      <x:c r="E27" s="59"/>
-      <x:c r="F27" s="59"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">r (ранг)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B28" s="63" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C28" s="59"/>
-      <x:c r="D28" s="59"/>
-      <x:c r="E28" s="59"/>
-      <x:c r="F28" s="59"/>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lora_alpha</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B29" s="63" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="C29" s="59"/>
-      <x:c r="D29" s="59"/>
-      <x:c r="E29" s="59"/>
-      <x:c r="F29" s="59"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="59"/>
-      <x:c r="B30" s="59"/>
-      <x:c r="C30" s="59"/>
-      <x:c r="D30" s="59"/>
-      <x:c r="E30" s="59"/>
-      <x:c r="F30" s="59"/>
-    </x:row>
-    <x:row r="31" ht="45" customHeight="1">
-      <x:c r="A31" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">целевой модуль</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B31" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">слоёв</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C31" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">вход</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D31" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">выход</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E31" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">параметров адаптера
-r × (вход + выход) × слоёв</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F31" s="56" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">включён?</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="59" t="str">
-        <x:v>q_proj</x:v>
-      </x:c>
-      <x:c r="B32" s="63" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C32" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="D32" s="63" t="n">
-        <x:v>2048</x:v>
-      </x:c>
-      <x:c r="E32" s="65" t="n">
-        <x:f>IF(OR(F32&lt;&gt;"да",COUNT(B32:D32)&lt;3),0,$B$28*(C32+D32)*B32)</x:f>
-        <x:v>1376256</x:v>
-      </x:c>
-      <x:c r="F32" s="63" t="str">
-        <x:v>да</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="59" t="str">
-        <x:v>k_proj</x:v>
-      </x:c>
-      <x:c r="B33" s="63" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C33" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="D33" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="E33" s="65" t="n">
-        <x:f>IF(OR(F33&lt;&gt;"да",COUNT(B33:D33)&lt;3),0,$B$28*(C33+D33)*B33)</x:f>
-        <x:v>917504</x:v>
-      </x:c>
-      <x:c r="F33" s="63" t="str">
-        <x:v>да</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="59" t="str">
-        <x:v>v_proj</x:v>
-      </x:c>
-      <x:c r="B34" s="63" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C34" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="D34" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="E34" s="65" t="n">
-        <x:f>IF(OR(F34&lt;&gt;"да",COUNT(B34:D34)&lt;3),0,$B$28*(C34+D34)*B34)</x:f>
-        <x:v>917504</x:v>
-      </x:c>
-      <x:c r="F34" s="63" t="str">
-        <x:v>да</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="59" t="str">
-        <x:v>o_proj</x:v>
-      </x:c>
-      <x:c r="B35" s="63" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C35" s="63" t="n">
-        <x:v>2048</x:v>
-      </x:c>
-      <x:c r="D35" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="E35" s="65" t="n">
-        <x:f>IF(OR(F35&lt;&gt;"да",COUNT(B35:D35)&lt;3),0,$B$28*(C35+D35)*B35)</x:f>
-        <x:v>1376256</x:v>
-      </x:c>
-      <x:c r="F35" s="63" t="str">
-        <x:v>да</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="59" t="str">
-        <x:v>gate_proj</x:v>
-      </x:c>
-      <x:c r="B36" s="63" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C36" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="D36" s="63" t="n">
-        <x:v>3072</x:v>
-      </x:c>
-      <x:c r="E36" s="65" t="n">
-        <x:f>IF(OR(F36&lt;&gt;"да",COUNT(B36:D36)&lt;3),0,$B$28*(C36+D36)*B36)</x:f>
-        <x:v>1835008</x:v>
-      </x:c>
-      <x:c r="F36" s="63" t="str">
-        <x:v>да</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="59" t="str">
-        <x:v>up_proj</x:v>
-      </x:c>
-      <x:c r="B37" s="63" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C37" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="D37" s="63" t="n">
-        <x:v>3072</x:v>
-      </x:c>
-      <x:c r="E37" s="65" t="n">
-        <x:f>IF(OR(F37&lt;&gt;"да",COUNT(B37:D37)&lt;3),0,$B$28*(C37+D37)*B37)</x:f>
-        <x:v>1835008</x:v>
-      </x:c>
-      <x:c r="F37" s="63" t="str">
-        <x:v>да</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="59" t="str">
-        <x:v>down_proj</x:v>
-      </x:c>
-      <x:c r="B38" s="63" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C38" s="63" t="n">
-        <x:v>3072</x:v>
-      </x:c>
-      <x:c r="D38" s="63" t="n">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="E38" s="65" t="n">
-        <x:f>IF(OR(F38&lt;&gt;"да",COUNT(B38:D38)&lt;3),0,$B$28*(C38+D38)*B38)</x:f>
-        <x:v>1835008</x:v>
-      </x:c>
-      <x:c r="F38" s="63" t="str">
-        <x:v>да</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="78" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">по вашей формуле</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B39" s="78"/>
-      <x:c r="C39" s="78"/>
-      <x:c r="D39" s="78"/>
-      <x:c r="E39" s="79" t="n">
-        <x:f>SUM(E32:E38)</x:f>
-        <x:v>10092544</x:v>
-      </x:c>
-      <x:c r="F39" s="78"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">что показал peft</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B40" s="59"/>
-      <x:c r="C40" s="59"/>
-      <x:c r="D40" s="59"/>
-      <x:c r="E40" s="64" t="n">
-        <x:v>10092544</x:v>
-      </x:c>
-      <x:c r="F40" s="59"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">совпало?</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B41" s="59"/>
-      <x:c r="C41" s="59"/>
-      <x:c r="D41" s="59"/>
-      <x:c r="E41" s="66" t="str">
-        <x:f>IF(E40="","заполните",IF(E39=E40,"да, совпало","НЕ СОВПАЛО"))</x:f>
-        <x:v>да, совпало</x:v>
-      </x:c>
-      <x:c r="F41" s="59"/>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="59"/>
-      <x:c r="B42" s="59"/>
-      <x:c r="C42" s="59"/>
-      <x:c r="D42" s="59"/>
-      <x:c r="E42" s="59"/>
-      <x:c r="F42" s="59"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">параметров базовой модели</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B43" s="59"/>
-      <x:c r="C43" s="59"/>
-      <x:c r="D43" s="59"/>
-      <x:c r="E43" s="64" t="n">
-        <x:v>596049920</x:v>
-      </x:c>
-      <x:c r="F43" s="59"/>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">доля обучаемых</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B44" s="59"/>
-      <x:c r="C44" s="59"/>
-      <x:c r="D44" s="59"/>
-      <x:c r="E44" s="77" t="n">
-        <x:f>IF(E43="","",E39/E43)</x:f>
-        <x:v>0.016932380428807035</x:v>
-      </x:c>
-      <x:c r="F44" s="59"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E17:E17">
@@ -2053,14 +1384,6 @@
     </x:cfRule>
     <x:cfRule type="expression" dxfId="1" priority="2">
       <x:formula>EXACT(E17,"да, совпало")</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="E41:E41">
-    <x:cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <x:formula>"да, совпало"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
-      <x:formula>"НЕ СОВПАЛО"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2071,8 +1394,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="43" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" customWidth="1"/>
+    <x:col min="2" max="2" width="34" customWidth="1"/>
     <x:col min="3" max="3" width="16" customWidth="1"/>
     <x:col min="4" max="4" width="12" customWidth="1"/>
     <x:col min="5" max="5" width="20" customWidth="1"/>
@@ -2098,8 +1421,10 @@
           <x:t xml:space="preserve">режим</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="6" t="str">
-        <x:v>пик, МиБ</x:v>
+      <x:c r="B4" s="6" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">пик, МБ</x:t>
+        </x:is>
       </x:c>
       <x:c r="C4" s="6" t="inlineStr">
         <x:is>
@@ -2123,15 +1448,15 @@
           <x:t xml:space="preserve">инференс</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="82" t="n">
-        <x:v>2525.6</x:v>
-      </x:c>
-      <x:c r="C5" s="83" t="n">
+      <x:c r="B5" s="18" t="n">
+        <x:v>2549.9</x:v>
+      </x:c>
+      <x:c r="C5" s="19" t="n">
         <x:f>IF($B$5="","",B5/$B$5)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D5" s="82" t="n">
-        <x:v>10.8</x:v>
+      <x:c r="D5" s="20" t="n">
+        <x:v>7.9</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
         <x:f>IF(OR(B5="",$B$14=""),"",IF(B5&gt;=$B$14,"да","МЕНЬШЕ ВЕСОВ"))</x:f>
@@ -2144,15 +1469,15 @@
           <x:t xml:space="preserve">full fine-tune</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="82" t="n">
-        <x:v>6809.3</x:v>
-      </x:c>
-      <x:c r="C6" s="83" t="n">
+      <x:c r="B6" s="18" t="n">
+        <x:v>6780.5</x:v>
+      </x:c>
+      <x:c r="C6" s="19" t="n">
         <x:f>IF($B$5="","",B6/$B$5)</x:f>
-        <x:v>2.696111815014254</x:v>
-      </x:c>
-      <x:c r="D6" s="82" t="n">
-        <x:v>22.4</x:v>
+        <x:v>2.6591238872112632</x:v>
+      </x:c>
+      <x:c r="D6" s="20" t="n">
+        <x:v>21.5</x:v>
       </x:c>
       <x:c r="E6" s="11" t="str">
         <x:f>IF(OR(B6="",$B$14=""),"",IF(B6&gt;=$B$14,"да","МЕНЬШЕ ВЕСОВ"))</x:f>
@@ -2165,15 +1490,15 @@
           <x:t xml:space="preserve">LoRA (r=8, q/v)</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" s="82" t="n">
-        <x:v>3291.1</x:v>
-      </x:c>
-      <x:c r="C7" s="83" t="n">
+      <x:c r="B7" s="18" t="n">
+        <x:v>3281.3</x:v>
+      </x:c>
+      <x:c r="C7" s="19" t="n">
         <x:f>IF($B$5="","",B7/$B$5)</x:f>
-        <x:v>1.3030962939499524</x:v>
-      </x:c>
-      <x:c r="D7" s="82" t="n">
-        <x:v>16.7</x:v>
+        <x:v>1.286834777834425</x:v>
+      </x:c>
+      <x:c r="D7" s="20" t="n">
+        <x:v>14.1</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
         <x:f>IF(OR(B7="",$B$14=""),"",IF(B7&gt;=$B$14,"да","МЕНЬШЕ ВЕСОВ"))</x:f>
@@ -2215,10 +1540,8 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="21" t="str">
-        <x:v>веса модели, МиБ</x:v>
-      </x:c>
-      <x:c r="B14" s="84" t="n">
+      <x:c r="A14" s="21" t="n"/>
+      <x:c r="B14" s="9" t="n">
         <x:f>IF(COUNT(B10:B11)&lt;2,"",B10*B11/1048576)</x:f>
         <x:v>1136.875</x:v>
       </x:c>
@@ -2231,82 +1554,82 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="80" t="inlineStr">
+      <x:c r="A17" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">устройство (cpu / cuda / mps)</x:t>
         </x:is>
       </x:c>
-      <x:c r="B17" s="81" t="str">
+      <x:c r="B17" s="22" t="str">
         <x:v>cpu</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="80" t="inlineStr">
+      <x:c r="A18" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">чем меряли память</x:t>
         </x:is>
       </x:c>
-      <x:c r="B18" s="81" t="str">
+      <x:c r="B18" s="22" t="str">
         <x:v>ru_maxrss</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="80" t="inlineStr">
+      <x:c r="A19" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">dtype</x:t>
         </x:is>
       </x:c>
-      <x:c r="B19" s="81" t="str">
+      <x:c r="B19" s="22" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="80" t="inlineStr">
+      <x:c r="A20" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">seq_len</x:t>
         </x:is>
       </x:c>
-      <x:c r="B20" s="81" t="n">
+      <x:c r="B20" s="22" t="n">
         <x:v>256</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="80" t="inlineStr">
+      <x:c r="A21" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">batch_size</x:t>
         </x:is>
       </x:c>
-      <x:c r="B21" s="81" t="n">
+      <x:c r="B21" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="80" t="inlineStr">
+      <x:c r="A22" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">сколько раз повторяли замер</x:t>
         </x:is>
       </x:c>
-      <x:c r="B22" s="81" t="n">
+      <x:c r="B22" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="48" customHeight="1">
-      <x:c r="A23" s="80" t="inlineStr">
+    <x:row r="23">
+      <x:c r="A23" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">что именно в шаге (forward / +backward / +optimizer)</x:t>
         </x:is>
       </x:c>
-      <x:c r="B23" s="81" t="str">
-        <x:v>Инференс: forward; обучение: forward + backward + шаг AdamW.</x:v>
+      <x:c r="B23" s="22" t="str">
+        <x:v>инференс: forward; full FT и LoRA: forward + backward + optimizer.step</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="80" t="inlineStr">
+      <x:c r="A24" s="17" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">модель</x:t>
         </x:is>
       </x:c>
-      <x:c r="B24" s="81" t="str">
+      <x:c r="B24" s="22" t="str">
         <x:v>Qwen/Qwen3-0.6B</x:v>
       </x:c>
     </x:row>
@@ -2367,68 +1690,68 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
-      <x:c r="A5" s="86" t="n">
+      <x:c r="A5" s="14" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B5" s="87" t="inlineStr">
+      <x:c r="B5" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Почему lm_head в вашей таблице весит столько, сколько весит?</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="88" t="str">
-        <x:v>lm_head имеет 0 собственных параметров: он использует те же 155 582 464 веса, что и embed. Общий тензор учитывается один раз.</x:v>
+      <x:c r="C5" s="24" t="str">
+        <x:v>lm_head весит 0 параметров: при tie_word_embeddings=True он использует тот же тензор, что и embed_tokens, поэтому второй раз вес не считается.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
-      <x:c r="A6" s="86" t="n">
+      <x:c r="A6" s="14" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B6" s="87" t="inlineStr">
+      <x:c r="B6" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Почему k_proj вдвое меньше q_proj?</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="88" t="str">
-        <x:v>У Q 16 голов по 128 чисел, а у K — 8. Поэтому q_proj: 2048 × 1024, k_proj: 1024 × 1024; число параметров различается вдвое.</x:v>
+      <x:c r="C6" s="24" t="str">
+        <x:v>В модели 16 голов запросов, но только 8 KV-голов. Поэтому выход q_proj равен 2048, а у k_proj — 1024, и параметров вдвое меньше.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
-      <x:c r="A7" s="86" t="n">
+      <x:c r="A7" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B7" s="87" t="inlineStr">
+      <x:c r="B7" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Почему MLP занимает большую долю модели, чем всё внимание вместе?</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="88" t="str">
-        <x:v>Три широкие матрицы MLP дают 264 241 152 параметра (44,34%). Четыре проекции attention дают 176 160 768 (29,56%): MLP больше в 1,5 раза.</x:v>
+      <x:c r="C7" s="24" t="str">
+        <x:v>В каждом из 28 блоков MLP содержит три большие матрицы с intermediate_size=3072. Вместе это 264 241 152 параметра против 176 160 768 у четырёх проекций внимания.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
-      <x:c r="A8" s="86" t="n">
+      <x:c r="A8" s="14" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B8" s="87" t="inlineStr">
+      <x:c r="B8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Почему при 0,192% обучаемых параметров LoRA экономит намного больше памяти, чем 0,192%?</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="88" t="str">
-        <x:v>Обучаются только 1 146 880 параметров адаптера. Для остальных не нужны градиенты и состояния AdamW: пик снижается с 6809.3 до 3291.1 МиБ; веса базы и активации остаются.</x:v>
+      <x:c r="C8" s="24" t="str">
+        <x:v>Для базовой модели LoRA не хранит градиенты и состояния AdamW. Поэтому при 0,192% обучаемых параметров пик снизился с 6780,5 до 3281,3 МБ; веса базы и активации всё равно остаются в памяти.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
-      <x:c r="A9" s="86" t="n">
+      <x:c r="A9" s="14" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B9" s="87" t="inlineStr">
+      <x:c r="B9" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Ваша метрика памяти — какая и почему именно она подходит вашему устройству?</x:t>
         </x:is>
       </x:c>
-      <x:c r="C9" s="88" t="str">
-        <x:v>Используется ru_maxrss: максимум RSS процесса за всё время. На CPU тензоры лежат в RAM; каждый режим запускается отдельным процессом, чтобы пики не смешивались.</x:v>
+      <x:c r="C9" s="24" t="str">
+        <x:v>Используется ru_maxrss: запуск идёт на CPU, тензоры лежат в обычной оперативной памяти, а эта метрика возвращает её пиковый расход процессом.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>